<commit_message>
Comment rows (#) in control sheets; fix template note-row trap
The shipped workbook's gray row-2 instruction notes were read as DATA by
the loader (a 100-char "parameter name" -> validation refusal). The loader
now skips any row whose first cell starts with '#', the template's note
rows are '#'-prefixed (and verified loader-safe in the round-trip check),
the suite's CSV test regression-guards the skip, and USER_GUIDE documents
comment rows + that PARAMETERS may be left empty.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/template/scenario_workbook.xlsx
+++ b/template/scenario_workbook.xlsx
@@ -104,7 +104,7 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -828,7 +828,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>scenario_id: letters/digits/underscore, max 24 chars (it becomes a folder name). parent_scenario runs the parent's steps first. Example rows below - replace with yours.</t>
+          <t># scenario_id: letters/digits/underscore, max 24 chars (it becomes a folder name). parent_scenario runs the parent's steps first. Example rows below - replace with yours.</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Steps run in step_no order (use 10, 20, 30 ... so you can insert later). where_clause / assignments / source are used literally - keep them Text-formatted. Example rows below - replace table and column names with your own.</t>
+          <t># Steps run in step_no order (use 10, 20, 30 ... so you can insert later). where_clause / assignments / source are used literally - keep them Text-formatted. Example rows below - replace table and column names with your own.</t>
         </is>
       </c>
     </row>
@@ -11083,7 +11083,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Reference as &amp;NAME in any where_clause / assignments / source cell. Blank scenario_id = global; a row with a scenario_id overrides the global for that scenario.</t>
+          <t># Reference as &amp;NAME in any where_clause / assignments / source cell. Blank scenario_id = global; a row with a scenario_id overrides the global for that scenario.</t>
         </is>
       </c>
     </row>

</xml_diff>